<commit_message>
Inject form version id in xml and force redownload of the form by adding the form_version version_id
</commit_message>
<xml_diff>
--- a/testdata/seed-data-command-event-tracker-form.xlsx
+++ b/testdata/seed-data-command-event-tracker-form.xlsx
@@ -63,7 +63,7 @@
     <t xml:space="preserve">is_existing</t>
   </si>
   <si>
-    <t xml:space="preserve">Existing kid ?</t>
+    <t xml:space="preserve">Existing kid SMS 2?</t>
   </si>
   <si>
     <t xml:space="preserve">text</t>
@@ -490,7 +490,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -512,12 +512,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -567,7 +561,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>

<commit_message>
Export events and and create relationships
</commit_message>
<xml_diff>
--- a/testdata/seed-data-command-event-tracker-form.xlsx
+++ b/testdata/seed-data-command-event-tracker-form.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="174">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -315,13 +315,19 @@
     <t xml:space="preserve">hh_repeat</t>
   </si>
   <si>
+    <t xml:space="preserve">hh_name</t>
+  </si>
+  <si>
     <t xml:space="preserve">What is the name of the household member?</t>
   </si>
   <si>
+    <t xml:space="preserve">hh_gender</t>
+  </si>
+  <si>
     <t xml:space="preserve">What is the gender of the household member?</t>
   </si>
   <si>
-    <t xml:space="preserve">age</t>
+    <t xml:space="preserve">hh_age</t>
   </si>
   <si>
     <t xml:space="preserve">What is the age of the household member?</t>
@@ -333,19 +339,19 @@
     <t xml:space="preserve">House hold address</t>
   </si>
   <si>
-    <t xml:space="preserve">street</t>
+    <t xml:space="preserve">hh_street</t>
   </si>
   <si>
     <t xml:space="preserve">Street</t>
   </si>
   <si>
-    <t xml:space="preserve">number</t>
+    <t xml:space="preserve">hh_number</t>
   </si>
   <si>
     <t xml:space="preserve">Number</t>
   </si>
   <si>
-    <t xml:space="preserve">city</t>
+    <t xml:space="preserve">hh_city</t>
   </si>
   <si>
     <t xml:space="preserve">City</t>
@@ -547,7 +553,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -577,12 +583,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -627,7 +627,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -646,10 +646,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1180,10 +1176,10 @@
         <v>14</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -1193,10 +1189,10 @@
         <v>20</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -1206,10 +1202,10 @@
         <v>24</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D47" s="1"/>
     </row>
@@ -1217,11 +1213,11 @@
       <c r="A48" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="5" t="s">
-        <v>101</v>
+      <c r="B48" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D48" s="1"/>
     </row>
@@ -1230,10 +1226,10 @@
         <v>14</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D49" s="1"/>
     </row>
@@ -1242,10 +1238,10 @@
         <v>14</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D50" s="1"/>
     </row>
@@ -1254,10 +1250,10 @@
         <v>14</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D51" s="1"/>
     </row>
@@ -1265,15 +1261,15 @@
       <c r="A52" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="5" t="s">
-        <v>101</v>
+      <c r="B52" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="1"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>96</v>
@@ -1308,7 +1304,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>1</v>
@@ -1319,453 +1315,453 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1773,10 +1769,10 @@
         <v>21</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1784,10 +1780,10 @@
         <v>21</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1816,18 +1812,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>